<commit_message>
Give each event edition its own activity and align sub-rubric labels with the event report
The Zumba na Caneca event summed the 2024, 2025 and 2026 editions because
all three shared one activity. Earlier editions now have their own
activities, which live only in the fixture lists so the downloadable
template keeps its four. The template instructions explain the rule. The
Apoio UPV and Apoio Junta sub-rubrics carry their full labels and the
reception performance description matches the handover document. The ledger
test asserts the Zumba and 20º CITADÃO totals with the event cutoff.
</commit_message>
<xml_diff>
--- a/fixtures/generated/invalid/checkpoint-mismatch.xlsx
+++ b/fixtures/generated/invalid/checkpoint-mismatch.xlsx
@@ -17,7 +17,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="84">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="82">
   <si>
     <t>Ficheiro de teste com erros propositados</t>
   </si>
@@ -124,7 +124,7 @@
     <t>Donativos</t>
   </si>
   <si>
-    <t>Apoio UPV</t>
+    <t>Apoio UPV (via AE ESAV)</t>
   </si>
   <si>
     <t>Zumba na Caneca</t>
@@ -133,10 +133,10 @@
     <t>Banco</t>
   </si>
   <si>
-    <t>Apoio Junta</t>
-  </si>
-  <si>
-    <t>18º CITADÃO</t>
+    <t>Apoio Junta de Freguesia</t>
+  </si>
+  <si>
+    <t>20º CITADÃO</t>
   </si>
   <si>
     <t>MB Way</t>
@@ -151,7 +151,7 @@
     <t>Inscrições e bilheteira</t>
   </si>
   <si>
-    <t>19º CITADÃO</t>
+    <t>Festivais</t>
   </si>
   <si>
     <t>TPA</t>
@@ -160,16 +160,10 @@
     <t>Bilheteira</t>
   </si>
   <si>
-    <t>20º CITADÃO</t>
-  </si>
-  <si>
     <t>Bar e merchandising</t>
   </si>
   <si>
     <t>Inscrições</t>
-  </si>
-  <si>
-    <t>Festivais</t>
   </si>
   <si>
     <t>Patrocínios</t>
@@ -1157,7 +1151,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>43</v>
       </c>
@@ -1173,13 +1167,10 @@
       <c r="F6" t="s">
         <v>43</v>
       </c>
-      <c r="H6" t="s">
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
         <v>47</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>48</v>
       </c>
       <c r="B7" t="s">
         <v>17</v>
@@ -1188,18 +1179,15 @@
         <v>31</v>
       </c>
       <c r="E7" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F7" t="s">
         <v>43</v>
       </c>
-      <c r="H7" t="s">
-        <v>50</v>
-      </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
         <v>17</v>
@@ -1208,15 +1196,15 @@
         <v>31</v>
       </c>
       <c r="E8" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F8" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="B9" t="s">
         <v>17</v>
@@ -1225,243 +1213,243 @@
         <v>31</v>
       </c>
       <c r="E9" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F9" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>53</v>
+      </c>
+      <c r="B10" t="s">
+        <v>54</v>
+      </c>
+      <c r="C10" t="s">
+        <v>31</v>
+      </c>
+      <c r="E10" t="s">
         <v>55</v>
       </c>
-      <c r="B10" t="s">
-        <v>56</v>
-      </c>
-      <c r="C10" t="s">
-        <v>31</v>
-      </c>
-      <c r="E10" t="s">
-        <v>57</v>
-      </c>
       <c r="F10" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="B11" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C11" t="s">
         <v>31</v>
       </c>
       <c r="E11" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F11" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="B12" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C12" t="s">
         <v>31</v>
       </c>
       <c r="E12" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F12" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B13" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C13" t="s">
         <v>31</v>
       </c>
       <c r="E13" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F13" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B14" t="s">
+        <v>54</v>
+      </c>
+      <c r="C14" t="s">
+        <v>31</v>
+      </c>
+      <c r="E14" t="s">
+        <v>63</v>
+      </c>
+      <c r="F14" t="s">
         <v>56</v>
-      </c>
-      <c r="C14" t="s">
-        <v>31</v>
-      </c>
-      <c r="E14" t="s">
-        <v>65</v>
-      </c>
-      <c r="F14" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="B15" t="s">
+        <v>54</v>
+      </c>
+      <c r="C15" t="s">
+        <v>31</v>
+      </c>
+      <c r="E15" t="s">
+        <v>65</v>
+      </c>
+      <c r="F15" t="s">
         <v>56</v>
-      </c>
-      <c r="C15" t="s">
-        <v>31</v>
-      </c>
-      <c r="E15" t="s">
-        <v>67</v>
-      </c>
-      <c r="F15" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B16" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C16" t="s">
         <v>31</v>
       </c>
       <c r="E16" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="F16" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B17" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C17" t="s">
         <v>31</v>
       </c>
       <c r="E17" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="F17" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B18" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C18" t="s">
         <v>31</v>
       </c>
       <c r="E18" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="F18" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="B19" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C19" t="s">
         <v>31</v>
       </c>
       <c r="E19" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="F19" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B20" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C20" t="s">
         <v>31</v>
       </c>
       <c r="E20" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="F20" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>76</v>
+      </c>
+      <c r="C21" t="s">
+        <v>77</v>
+      </c>
+      <c r="E21" t="s">
         <v>78</v>
       </c>
-      <c r="C21" t="s">
-        <v>79</v>
-      </c>
-      <c r="E21" t="s">
-        <v>80</v>
-      </c>
       <c r="F21" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="22" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E22" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="F22" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
     </row>
     <row r="23" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E23" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F23" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E24" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="F24" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
     <row r="25" spans="5:6" x14ac:dyDescent="0.25">
       <c r="E25" t="s">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F25" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
     </row>
   </sheetData>

</xml_diff>